<commit_message>
Chages in code both side YOuth and Creater
</commit_message>
<xml_diff>
--- a/resources/Event_Name.xlsx
+++ b/resources/Event_Name.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="49">
   <si>
     <t>Event_Name</t>
   </si>
@@ -147,6 +147,18 @@
   </si>
   <si>
     <t>Swachhta Hi Seva Prayagraj</t>
+  </si>
+  <si>
+    <t>Bhopal Swachhta Hi Seva</t>
+  </si>
+  <si>
+    <t>Ahmedabad Swachhta Hi Seva</t>
+  </si>
+  <si>
+    <t>Varanasi Swachhta Hi Seva</t>
+  </si>
+  <si>
+    <t>Prayagraj Swachhta Hi Seva</t>
   </si>
 </sst>
 </file>
@@ -191,7 +203,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A54"/>
+  <dimension ref="A1:A59"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -464,6 +476,31 @@
         <v>31</v>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="s" s="0">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s" s="0">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s" s="0">
+        <v>48</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
changes evevt name and counter and youth
</commit_message>
<xml_diff>
--- a/resources/Event_Name.xlsx
+++ b/resources/Event_Name.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="57">
   <si>
     <t>Event_Name</t>
   </si>
@@ -180,6 +180,9 @@
   </si>
   <si>
     <t>Nagpur Swachhta Hi Seva</t>
+  </si>
+  <si>
+    <t>Noida Swachhta Hi Seva</t>
   </si>
 </sst>
 </file>
@@ -224,7 +227,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A69"/>
+  <dimension ref="A1:A70"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -572,6 +575,11 @@
         <v>55</v>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="s" s="0">
+        <v>56</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>